<commit_message>
n8n board refresh 2026-09-09T17:44:25Z
</commit_message>
<xml_diff>
--- a/app/reports/ENOV_research.xlsx
+++ b/app/reports/ENOV_research.xlsx
@@ -620,7 +620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-07 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-09-09 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>18.56</v>
+        <v>19.1</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>0.04783999919891357</v>
+        <v>0.04835000038146973</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B35" s="20" t="n">
-        <v>57669493.10344828</v>
+        <v>57669495.28795811</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="B37" s="22" t="n">
-        <v>18.56</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="38">
@@ -1508,14 +1508,14 @@
         </is>
       </c>
       <c r="C5" s="30" t="n">
-        <v>1070345792</v>
+        <v>1101487360</v>
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31" t="n">
-        <v>6.41</v>
+        <v>6.62</v>
       </c>
       <c r="F5" s="31" t="n">
-        <v>1.06</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="6">
@@ -1531,13 +1531,13 @@
       </c>
       <c r="C6" s="32" t="n"/>
       <c r="D6" s="33" t="n">
-        <v>23.644156</v>
+        <v>23.28052</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>16.289</v>
+        <v>16.283</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>2.994</v>
+        <v>2.993</v>
       </c>
     </row>
     <row r="7">
@@ -1552,16 +1552,16 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>1924621952</v>
+        <v>1875655808</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>21.21591</v>
+        <v>20.676136</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>12.724</v>
+        <v>12.622</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>3.12</v>
+        <v>3.095</v>
       </c>
     </row>
     <row r="8">
@@ -1576,16 +1576,16 @@
         </is>
       </c>
       <c r="C8" s="32" t="n">
-        <v>4410535936</v>
+        <v>4382240256</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>28.666668</v>
+        <v>28.48276</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>13.093</v>
+        <v>13.014</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>2.091</v>
+        <v>2.079</v>
       </c>
     </row>
     <row r="9">
@@ -1600,16 +1600,16 @@
         </is>
       </c>
       <c r="C9" s="32" t="n">
-        <v>1030276736</v>
+        <v>1030628864</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>85.223305</v>
+        <v>85.252426</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>41.067</v>
+        <v>41.525</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>3.868</v>
+        <v>3.911</v>
       </c>
     </row>
     <row r="10">
@@ -1624,16 +1624,16 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>1989747712</v>
+        <v>1969676032</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>31.78903</v>
+        <v>31.468357</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>16.676</v>
+        <v>16.706</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>3.164</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="11">
@@ -1648,16 +1648,16 @@
         </is>
       </c>
       <c r="C11" s="32" t="n">
-        <v>2359920384</v>
+        <v>2334548224</v>
       </c>
       <c r="D11" s="33" t="n">
-        <v>33.46729</v>
+        <v>33.107475</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>15.014</v>
+        <v>14.977</v>
       </c>
       <c r="F11" s="33" t="n">
-        <v>2.965</v>
+        <v>2.957</v>
       </c>
     </row>
     <row r="12">
@@ -1672,14 +1672,14 @@
         </is>
       </c>
       <c r="C12" s="32" t="n">
-        <v>148890640</v>
+        <v>145166768</v>
       </c>
       <c r="D12" s="33" t="n"/>
       <c r="E12" s="33" t="n">
-        <v>-33.62</v>
+        <v>-32.395</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>0.582</v>
+        <v>0.5610000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1694,16 +1694,16 @@
         </is>
       </c>
       <c r="C13" s="32" t="n">
-        <v>16494090240</v>
+        <v>16604669952</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>32.146553</v>
+        <v>32.408634</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>18.35</v>
+        <v>18.496</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>4.953</v>
+        <v>4.992</v>
       </c>
     </row>
     <row r="15">

</xml_diff>